<commit_message>
adding formula reference card slide
</commit_message>
<xml_diff>
--- a/MATH/M01/bus123-math-m01-l01-starter.xlsx
+++ b/MATH/M01/bus123-math-m01-l01-starter.xlsx
@@ -2,9 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="25600" windowHeight="15240" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live You Try It" sheetId="2" state="visible" r:id="rId2"/>
@@ -12,20 +9,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormulaReferenceCard" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -58,10 +52,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color rgb="FF1A1F2C"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -81,8 +73,20 @@
       <color rgb="FF355773"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFB8843D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF355773"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -139,15 +143,49 @@
         <fgColor rgb="FFB8843D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0E1116"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF3EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2EEE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0E1116"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF3EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2EEE5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin">
         <color rgb="FFE5E1D6"/>
@@ -161,7 +199,6 @@
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -176,21 +213,16 @@
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FFE5E1D6"/>
       </top>
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FFE5E1D6"/>
       </right>
@@ -200,82 +232,56 @@
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FFE5E1D6"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FFE5E1D6"/>
       </right>
       <top style="thin">
         <color rgb="FFE5E1D6"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF4A7C5E"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FFE5E1D6"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color rgb="FF4A7C5E"/>
       </left>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FFE5E1D6"/>
       </right>
-      <top/>
       <bottom style="thin">
         <color rgb="FFE5E1D6"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -379,41 +385,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4CCCC"/>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4CCCC"/>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -486,7 +532,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -528,72 +574,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -649,7 +637,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -658,13 +646,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -698,17 +686,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -763,8 +740,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -772,7 +747,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
@@ -794,8 +769,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="20">
       <c r="A5" s="26" t="inlineStr">
         <is>
@@ -803,7 +776,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="24" customHeight="1" s="20">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -864,8 +836,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="24" customHeight="1" s="20">
       <c r="A14" s="26" t="inlineStr">
         <is>
@@ -873,7 +843,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="28" customHeight="1" s="20">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -946,8 +915,6 @@
       <c r="G19" s="23" t="n"/>
       <c r="H19" s="24" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22" ht="24" customHeight="1" s="20">
       <c r="A22" s="27" t="inlineStr">
         <is>
@@ -955,7 +922,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
@@ -981,8 +947,7 @@
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A24:H25"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1017,8 +982,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1" s="20">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -1349,7 +1312,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="16" customHeight="1" s="20">
       <c r="A18" s="29" t="inlineStr">
         <is>
@@ -1357,7 +1319,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
         <is>
@@ -1402,7 +1363,7 @@
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1410,7 +1371,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
@@ -1437,8 +1398,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="20">
       <c r="A5" s="26" t="inlineStr">
         <is>
@@ -1446,7 +1405,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="28" customHeight="1" s="20">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -1765,8 +1723,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="24" customHeight="1" s="20">
       <c r="A18" s="27" t="inlineStr">
         <is>
@@ -1774,7 +1730,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="28" customHeight="1" s="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -2093,8 +2048,7 @@
       <formula>OR(ISNUMBER(SEARCH("Try",F8)),ISNUMBER(SEARCH("Check",F8)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2102,469 +2056,169 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="20" min="1" max="1"/>
-    <col width="34" customWidth="1" style="20" min="2" max="2"/>
-    <col width="46" customWidth="1" style="20" min="3" max="3"/>
-    <col width="36" customWidth="1" style="20" min="4" max="4"/>
+    <col width="21.11000061035156" customWidth="1" style="20" min="1" max="1"/>
+    <col width="25.55999946594238" customWidth="1" style="20" min="2" max="2"/>
+    <col width="34.43999862670898" customWidth="1" style="20" min="3" max="3"/>
+    <col width="33.33000183105469" customWidth="1" style="20" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="20">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>Formula Reference Card · BUS123 MATH-M01</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1" s="20">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Use this as a syntax reminder, then return to the yellow cells.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4" ht="24" customHeight="1" s="20">
-      <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>ARITHMETIC OPERATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1" s="20">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="1" ht="31.5" customHeight="1" s="20">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>Concept</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Excel Syntax</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Use It For</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>Excel Pattern</t>
+        </is>
+      </c>
+      <c r="C1" s="54" t="inlineStr">
+        <is>
+          <t>Plain-English Meaning</t>
+        </is>
+      </c>
+      <c r="D1" s="54" t="inlineStr">
         <is>
           <t>Watch Out For</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1" s="20">
-      <c r="A6" s="25" t="inlineStr">
+    <row r="2" ht="31.5" customHeight="1" s="20">
+      <c r="A2" s="58" t="inlineStr">
         <is>
           <t>Addition range</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>'=SUM(B2:B10)</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>Adds a range</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>Do not type every number if a range exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1" s="20">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>=SUM(B2:B10)</t>
+        </is>
+      </c>
+      <c r="C2" s="58" t="inlineStr">
+        <is>
+          <t>Adds a column or row of related numbers.</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t>Do not type every number if a range exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31.5" customHeight="1" s="20">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Subtraction</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>'=B5-C5</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="inlineStr">
-        <is>
-          <t>Difference between two cells</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>Check units</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1" s="20">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>=B5-C5</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="inlineStr">
+        <is>
+          <t>Finds the difference between two cells.</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Check that both cells use the same units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31.5" customHeight="1" s="20">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>Multiplication</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>'=B3*C3</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
-        <is>
-          <t>Quantity times fee/rate</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>Check time period</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1" s="20">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>=B3*C3</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Multiplies quantity by fee, rate, or price.</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>Check the time period before multiplying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31.5" customHeight="1" s="20">
+      <c r="A5" s="58" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>'=B7/C7</t>
-        </is>
-      </c>
-      <c r="C9" s="22" t="inlineStr">
-        <is>
-          <t>Total divided by count</t>
-        </is>
-      </c>
-      <c r="D9" s="22" t="inlineStr">
-        <is>
-          <t>Denominator cannot be zero</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11" ht="24" customHeight="1" s="20">
-      <c r="A11" s="27" t="inlineStr">
-        <is>
-          <t>FRACTIONS &amp; RATIOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1" s="20">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Excel Syntax</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Use It For</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Watch Out For</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1" s="20">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>Fraction to decimal</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>'=B2/C2</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="inlineStr">
-        <is>
-          <t>Numerator divided by denominator</t>
-        </is>
-      </c>
-      <c r="D13" s="22" t="inlineStr">
-        <is>
-          <t>Denominator is the whole</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1" s="20">
-      <c r="A14" s="25" t="inlineStr">
-        <is>
-          <t>Fraction as percent</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>'=B2/C2</t>
-        </is>
-      </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t>Same formula, formatted as %</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
-        <is>
-          <t>Do not multiply by 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1" s="20">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t>Part of total</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>'=part/whole</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="inlineStr">
-        <is>
-          <t>Share of a total</t>
-        </is>
-      </c>
-      <c r="D15" s="22" t="inlineStr">
-        <is>
-          <t>Use current total</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17" ht="24" customHeight="1" s="20">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>PERCENT CALCULATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1" s="20">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Excel Syntax</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Use It For</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Watch Out For</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1" s="20">
-      <c r="A19" s="22" t="inlineStr">
-        <is>
-          <t>% of a whole</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>'=B4*B5</t>
-        </is>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
-        <is>
-          <t>Whole times rate</t>
-        </is>
-      </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Rate as decimal or percent</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1" s="20">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>Grow by X%</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>'=B4*(1+B5)</t>
-        </is>
-      </c>
-      <c r="C20" s="25" t="inlineStr">
-        <is>
-          <t>Base increased by rate</t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="inlineStr">
-        <is>
-          <t>Use 1 + rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1" s="20">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>% change</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>'=(new-old)/old</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>Change over time</t>
-        </is>
-      </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Old value is the denominator</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1" s="20">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>Ratio as %</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>'=part/whole</t>
-        </is>
-      </c>
-      <c r="C22" s="25" t="inlineStr">
-        <is>
-          <t>Share at one point in time</t>
-        </is>
-      </c>
-      <c r="D22" s="25" t="inlineStr">
-        <is>
-          <t>Different from percent change</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24" ht="24" customHeight="1" s="20">
-      <c r="A24" s="34" t="inlineStr">
-        <is>
-          <t>COMMON MISTAKES</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1" s="20">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Excel Syntax</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Use It For</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Watch Out For</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1" s="20">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>Unit mismatch</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Label units in headers</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>Quarterly vs annual, dollars vs cents</t>
-        </is>
-      </c>
-      <c r="D26" s="25" t="inlineStr">
-        <is>
-          <t>Excel will not warn you</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1" s="20">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>Wrong base</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>'=(new-old)/old</t>
-        </is>
-      </c>
-      <c r="C27" s="22" t="inlineStr">
-        <is>
-          <t>Base is older number</t>
-        </is>
-      </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>Do not divide by new value</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1" s="20">
-      <c r="A28" s="25" t="inlineStr">
-        <is>
-          <t>Hardcoded values</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>'=B2*B3</t>
-        </is>
-      </c>
-      <c r="C28" s="25" t="inlineStr">
-        <is>
-          <t>Reference cells so formulas update</t>
-        </is>
-      </c>
-      <c r="D28" s="25" t="inlineStr">
-        <is>
-          <t>Avoid =57*4200 when cells exist</t>
-        </is>
-      </c>
-    </row>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>=B7/C7</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>Splits a total across a count or base.</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>The denominator cannot be zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31.5" customHeight="1" s="20">
+      <c r="A6" s="58" t="inlineStr">
+        <is>
+          <t>Percent share</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>=B2/C2</t>
+        </is>
+      </c>
+      <c r="C6" s="58" t="inlineStr">
+        <is>
+          <t>Shows a part as a share of the whole.</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>Format as percent instead of multiplying by 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1" s="20"/>
+    <row r="8" ht="34" customHeight="1" s="20"/>
+    <row r="9" ht="34" customHeight="1" s="20"/>
+    <row r="11" ht="24" customHeight="1" s="20"/>
+    <row r="12" ht="28" customHeight="1" s="20"/>
+    <row r="13" ht="34" customHeight="1" s="20"/>
+    <row r="14" ht="34" customHeight="1" s="20"/>
+    <row r="15" ht="34" customHeight="1" s="20"/>
+    <row r="17" ht="24" customHeight="1" s="20"/>
+    <row r="18" ht="28" customHeight="1" s="20"/>
+    <row r="19" ht="34" customHeight="1" s="20"/>
+    <row r="20" ht="34" customHeight="1" s="20"/>
+    <row r="21" ht="34" customHeight="1" s="20"/>
+    <row r="22" ht="34" customHeight="1" s="20"/>
+    <row r="24" ht="24" customHeight="1" s="20"/>
+    <row r="25" ht="28" customHeight="1" s="20"/>
+    <row r="26" ht="34" customHeight="1" s="20"/>
+    <row r="27" ht="34" customHeight="1" s="20"/>
+    <row r="28" ht="34" customHeight="1" s="20"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>